<commit_message>
feat: 多主题切换 + PPT 视觉优化 + Bug 修复 (v2.12.1)
v2.12.1 多主题 & 视觉优化:
- 新增 11 套预设配色主题（基于 PPT Generator Skill）
  - 默认/午夜商务/科技深空/珊瑚活力/暖陶简约/海洋渐变/炭灰极简/青绿信任/莓果奶油/鼠尾草静/樱桃大胆
- PptTheme 支持 theme_name 参数 + from_config 支持主题名
- PPT 配置 Sheet 表头前加"主题|珊瑚活力"即可切换
- 新增 get_theme_preset() 和 list_theme_names() 工具函数

视觉增强:
- 封面: 主题色装饰几何圆点 + 底部装饰条
- 章节页: 左上角装饰块 + 右下角微细圆点
- 结尾页: 对称装饰圆点
- 结论卡片: 背景/边框色跟随主题
- 页面标题左侧竖条加宽

Bug 修复:
- _parse_mapping 不再将 val_map_str 作为列映射（误改了值字段名）
- collect_task_scalars numpy.int64 改用 float() 转换（isinstance 误判）
- _read_sheet_data 多区块 Sheet 只取第一区块，避免数据覆盖

excel_reader:
- _find_or_get_sheet 检查前3行，支持键值行在表头之上

防护用例全部通过。
</commit_message>
<xml_diff>
--- a/cases/00_防护用例/项目配置.xlsx
+++ b/cases/00_防护用例/项目配置.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1337,6 +1337,116 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>测试数据.xlsx</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>销售明细</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>销售额</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>历史标量</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>总销售额</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>标量生产者</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>测试数据.xlsx</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>销售明细</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>地区</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>销量</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>按地区汇总</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>地区销量</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>销量/总销售额=销量占比</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>标量消费者</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1348,7 +1458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1368,120 +1478,102 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>珊瑚活力</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>页码</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>页面类型</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>页面标题</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>布局</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>图表类型</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>数据Sheet</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>X轴</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>Y轴</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>图表标题</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>区块名</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>结论模板</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>数据源</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
         <is>
           <t>是否生成</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N2" s="1" t="inlineStr">
         <is>
           <t>文字内容</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="3">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>封面</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>销售数据分析报告
 防护用例|基础防护测试 | 全特性覆盖</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>目录</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>目录</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -1502,16 +1594,16 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>章节</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>一、销售汇总分析|各地区销售数据多维分析</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -1532,59 +1624,27 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>内容</t>
+          <t>章节</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>各地区销售汇总</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>1图</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>按地区汇总</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>地区</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>总销售额</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>各地区总销售额</t>
-        </is>
-      </c>
+          <t>一、销售汇总分析|各地区销售数据多维分析</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>销售额最高地区: {max_cat} ({max_val})</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>透视结果</t>
-        </is>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -1594,95 +1654,117 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>各地区销售汇总</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1图</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>按地区汇总</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>地区</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>总销售额</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>各地区总销售额</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>销售额最高地区: {max_cat} ({max_val})</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>透视结果</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>多维统计分析</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2图左右</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>bar</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>地区多维统计</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>地区</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>总销售额</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>各地区销售额对比</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>透视结果</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>pie</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>地区占比</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>地区</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>销售额占比</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>各地区销售额占比</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>透视结果</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -1691,60 +1773,38 @@
       <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>内容</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>销售额分箱分布</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>1图</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>pie</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>销售额分箱</t>
+          <t>地区占比</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>销售额区间</t>
+          <t>地区</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>客户数</t>
+          <t>销售额占比</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>销售额区间客户分布</t>
+          <t>各地区销售额占比</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>共 {count} 个区间</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>透视结果</t>
-        </is>
-      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -1754,41 +1814,103 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>销售额分箱分布</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1图</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>销售额分箱</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>销售额区间</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>客户数</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>销售额区间客户分布</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>共 {count} 个区间</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>透视结果</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>分析结论与说明</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>左图右文</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>本报告由防护用例自动生成</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>本报告基于测试数据生成，覆盖以下特性：
 1. 透视分析（分组、交叉表、占比、分箱）
@@ -1800,91 +1922,61 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>内容</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>block合并测试</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>1图</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>block合并测试</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>销售额区间</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>客户数_A</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>block合并测试(列A)</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>验证行维度不同+映射相同=合并区块</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>透视结果</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr"/>
-    </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>章节</t>
+          <t>内容</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>二、扩展测试|长标签与布局验证</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+          <t>block合并测试</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1图</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>block合并测试</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>销售额区间</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>客户数_A</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>block合并测试(列A)</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>验证行维度不同+映射相同=合并区块</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>透视结果</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -1894,59 +1986,27 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>内容</t>
+          <t>章节</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>城市销售长标签测试</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>1图</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>城市销售</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>城市</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>销售额</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>各城市销售额对比</t>
-        </is>
-      </c>
+          <t>二、扩展测试|长标签与布局验证</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>销售额最高城市: {max_cat} ({max_val})</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>测试数据.xlsx</t>
-        </is>
-      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -1956,27 +2016,59 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>结尾</t>
+          <t>内容</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>谢谢|防护用例测试完成</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+          <t>城市销售长标签测试</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>1图</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>城市销售</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>城市</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>销售额</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>各城市销售额对比</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>销售额最高城市: {max_cat} ({max_val})</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>测试数据.xlsx</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -1986,61 +2078,91 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>内容</t>
+          <t>结尾</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>跳过测试页(不应生成)</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>1图</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>按地区汇总</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>地区</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>总销售额</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>不应出现的图表</t>
-        </is>
-      </c>
+          <t>谢谢|防护用例测试完成</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>跳过测试页(不应生成)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>1图</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>按地区汇总</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>地区</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>总销售额</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>不应出现的图表</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>透视结果</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>